<commit_message>
Created BV Tuning Optimizer
</commit_message>
<xml_diff>
--- a/BVSimulationFiles/109.xlsx
+++ b/BVSimulationFiles/109.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1 Copy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1 Copy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1 Copy Copy" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -414,75 +414,60 @@
         <v>0</v>
       </c>
       <c r="C1" t="n">
-        <v>0.001541666666666667</v>
+        <v>0.001947368421052632</v>
       </c>
       <c r="D1" t="n">
-        <v>0.003083333333333334</v>
+        <v>0.003894736842105264</v>
       </c>
       <c r="E1" t="n">
-        <v>0.004625000000000001</v>
+        <v>0.005842105263157896</v>
       </c>
       <c r="F1" t="n">
-        <v>0.006166666666666668</v>
+        <v>0.007789473684210528</v>
       </c>
       <c r="G1" t="n">
-        <v>0.007708333333333334</v>
+        <v>0.00973684210526316</v>
       </c>
       <c r="H1" t="n">
-        <v>0.009250000000000001</v>
+        <v>0.01168421052631579</v>
       </c>
       <c r="I1" t="n">
-        <v>0.01079166666666667</v>
+        <v>0.01363157894736842</v>
       </c>
       <c r="J1" t="n">
-        <v>0.01233333333333334</v>
+        <v>0.01557894736842106</v>
       </c>
       <c r="K1" t="n">
-        <v>0.013875</v>
+        <v>0.01752631578947369</v>
       </c>
       <c r="L1" t="n">
-        <v>0.01541666666666667</v>
+        <v>0.01947368421052632</v>
       </c>
       <c r="M1" t="n">
-        <v>0.01695833333333334</v>
+        <v>0.02142105263157895</v>
       </c>
       <c r="N1" t="n">
-        <v>0.0185</v>
+        <v>0.02336842105263158</v>
       </c>
       <c r="O1" t="n">
-        <v>0.02004166666666667</v>
+        <v>0.02531578947368422</v>
       </c>
       <c r="P1" t="n">
-        <v>0.02158333333333334</v>
+        <v>0.02726315789473685</v>
       </c>
       <c r="Q1" t="n">
-        <v>0.023125</v>
+        <v>0.02921052631578948</v>
       </c>
       <c r="R1" t="n">
-        <v>0.02466666666666667</v>
+        <v>0.03115789473684211</v>
       </c>
       <c r="S1" t="n">
-        <v>0.02620833333333334</v>
+        <v>0.03310526315789474</v>
       </c>
       <c r="T1" t="n">
-        <v>0.02775</v>
+        <v>0.03505263157894738</v>
       </c>
       <c r="U1" t="n">
-        <v>0.02929166666666667</v>
-      </c>
-      <c r="V1" t="n">
-        <v>0.03083333333333334</v>
-      </c>
-      <c r="W1" t="n">
-        <v>0.032375</v>
-      </c>
-      <c r="X1" t="n">
-        <v>0.03391666666666667</v>
-      </c>
-      <c r="Y1" t="n">
-        <v>0.03545833333333334</v>
-      </c>
-      <c r="Z1" t="n">
         <v>0.03700000000000001</v>
       </c>
     </row>

</xml_diff>